<commit_message>
feat: notes tambahan after bimbingan
</commit_message>
<xml_diff>
--- a/Experiments/January17th/Summarization.xlsx
+++ b/Experiments/January17th/Summarization.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10814"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\personal\prethesis-experiments\Experiments\January17th\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/williamchristian/Documents/PersonalProjects/prethesis-experiments/Experiments/January17th/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13C574F7-0B50-47A4-BE70-8BE94AFB0E2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15C6B6BC-4A38-5C4A-9C05-8B262540B818}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13290" xr2:uid="{A7E435C2-3E53-4AA9-B99C-2C8358D38639}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{A7E435C2-3E53-4AA9-B99C-2C8358D38639}"/>
   </bookViews>
   <sheets>
     <sheet name="Supervised Learning" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="22">
   <si>
     <t>DistilBERT</t>
   </si>
@@ -93,6 +93,15 @@
   </si>
   <si>
     <t>Emotion</t>
+  </si>
+  <si>
+    <t>confusion matrix</t>
+  </si>
+  <si>
+    <t>training, test,validation review</t>
+  </si>
+  <si>
+    <t>augmentasi</t>
   </si>
 </sst>
 </file>
@@ -174,9 +183,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -184,6 +190,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -754,64 +763,64 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{199E1B80-8EC0-43B2-8FA2-B5F9B938102D}" name="Table1" displayName="Table1" ref="B3:H10" totalsRowShown="0" headerRowDxfId="28" dataDxfId="27">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{199E1B80-8EC0-43B2-8FA2-B5F9B938102D}" name="Table1" displayName="Table1" ref="B3:H10" totalsRowShown="0" headerRowDxfId="35" dataDxfId="34">
   <autoFilter ref="B3:H10" xr:uid="{199E1B80-8EC0-43B2-8FA2-B5F9B938102D}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{DCC6D35F-D5EF-46AD-9FD6-49FCC7AC28A0}" name="Dataset Name" dataDxfId="35"/>
-    <tableColumn id="2" xr3:uid="{70E59C2A-2EDB-4C14-9BAF-EB33706168E3}" name="Accuracy" dataDxfId="34"/>
-    <tableColumn id="3" xr3:uid="{EDC30577-A39D-4350-9191-12C5D20B220F}" name="Precision" dataDxfId="33"/>
-    <tableColumn id="4" xr3:uid="{E758F08B-56D3-4AA7-8E95-A7438AEDFBD9}" name="Recall" dataDxfId="32"/>
-    <tableColumn id="5" xr3:uid="{005125B9-D24C-4AEF-98B1-597916E8F957}" name="F1" dataDxfId="31"/>
-    <tableColumn id="6" xr3:uid="{76D8407A-C5E5-4C77-A405-E0905CFE9FEA}" name="Loss" dataDxfId="30"/>
-    <tableColumn id="7" xr3:uid="{D237F0C4-A361-4C57-BF94-14C88D159A46}" name="Epoch" dataDxfId="29"/>
+    <tableColumn id="1" xr3:uid="{DCC6D35F-D5EF-46AD-9FD6-49FCC7AC28A0}" name="Dataset Name" dataDxfId="33"/>
+    <tableColumn id="2" xr3:uid="{70E59C2A-2EDB-4C14-9BAF-EB33706168E3}" name="Accuracy" dataDxfId="32"/>
+    <tableColumn id="3" xr3:uid="{EDC30577-A39D-4350-9191-12C5D20B220F}" name="Precision" dataDxfId="31"/>
+    <tableColumn id="4" xr3:uid="{E758F08B-56D3-4AA7-8E95-A7438AEDFBD9}" name="Recall" dataDxfId="30"/>
+    <tableColumn id="5" xr3:uid="{005125B9-D24C-4AEF-98B1-597916E8F957}" name="F1" dataDxfId="29"/>
+    <tableColumn id="6" xr3:uid="{76D8407A-C5E5-4C77-A405-E0905CFE9FEA}" name="Loss" dataDxfId="28"/>
+    <tableColumn id="7" xr3:uid="{D237F0C4-A361-4C57-BF94-14C88D159A46}" name="Epoch" dataDxfId="27"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E01C6D3D-B089-4590-80B9-1C881116497F}" name="Table13" displayName="Table13" ref="J12:P17" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
-  <autoFilter ref="J12:P17" xr:uid="{E01C6D3D-B089-4590-80B9-1C881116497F}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E01C6D3D-B089-4590-80B9-1C881116497F}" name="Table13" displayName="Table13" ref="J12:P20" totalsRowShown="0" headerRowDxfId="26" dataDxfId="25">
+  <autoFilter ref="J12:P20" xr:uid="{E01C6D3D-B089-4590-80B9-1C881116497F}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{AB72BE09-8692-48E6-B7DE-A6BC3FF26E73}" name="Dataset Name" dataDxfId="26"/>
-    <tableColumn id="2" xr3:uid="{1B096B93-D180-4C5B-9EA7-7F01F74609E7}" name="Accuracy" dataDxfId="25"/>
-    <tableColumn id="3" xr3:uid="{0241CD65-36BB-47D0-9C7A-29619EF541D0}" name="Precision" dataDxfId="24"/>
-    <tableColumn id="4" xr3:uid="{1F21A8FF-84F9-48D1-B6CA-59115C30C8AF}" name="Recall" dataDxfId="23"/>
-    <tableColumn id="5" xr3:uid="{221D1CE2-60E2-400C-B768-BB11E227767E}" name="F1" dataDxfId="22"/>
-    <tableColumn id="6" xr3:uid="{2AAB4399-2F4E-4B01-9577-E412F80D17FD}" name="Loss" dataDxfId="21"/>
-    <tableColumn id="7" xr3:uid="{5F0D1A2A-30C1-4B38-B066-A83BFFEE7FF0}" name="Epoch" dataDxfId="20"/>
+    <tableColumn id="1" xr3:uid="{AB72BE09-8692-48E6-B7DE-A6BC3FF26E73}" name="Dataset Name" dataDxfId="24"/>
+    <tableColumn id="2" xr3:uid="{1B096B93-D180-4C5B-9EA7-7F01F74609E7}" name="Accuracy" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{0241CD65-36BB-47D0-9C7A-29619EF541D0}" name="Precision" dataDxfId="22"/>
+    <tableColumn id="4" xr3:uid="{1F21A8FF-84F9-48D1-B6CA-59115C30C8AF}" name="Recall" dataDxfId="21"/>
+    <tableColumn id="5" xr3:uid="{221D1CE2-60E2-400C-B768-BB11E227767E}" name="F1" dataDxfId="20"/>
+    <tableColumn id="6" xr3:uid="{2AAB4399-2F4E-4B01-9577-E412F80D17FD}" name="Loss" dataDxfId="19"/>
+    <tableColumn id="7" xr3:uid="{5F0D1A2A-30C1-4B38-B066-A83BFFEE7FF0}" name="Epoch" dataDxfId="18"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{115431F0-BE93-4ADF-89A6-0E800D823C2F}" name="Table134" displayName="Table134" ref="B21:H28" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{115431F0-BE93-4ADF-89A6-0E800D823C2F}" name="Table134" displayName="Table134" ref="B21:H28" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16">
   <autoFilter ref="B21:H28" xr:uid="{115431F0-BE93-4ADF-89A6-0E800D823C2F}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{6DA5A62F-F191-4700-A4DA-1ECCC0798408}" name="Dataset Name" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{6229C568-365F-4FB5-B5A5-14F4C8640478}" name="Accuracy" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{75BF09EF-9AEE-4394-90C3-0A038B9B0213}" name="Precision" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{4B15F953-1DB4-400F-816B-C322B01A4C96}" name="Recall" dataDxfId="14"/>
-    <tableColumn id="5" xr3:uid="{F8BED74C-48BE-4570-B328-816EDC50C33B}" name="F1" dataDxfId="13"/>
-    <tableColumn id="6" xr3:uid="{09327258-5F58-4797-9AC7-3B966B9FB96D}" name="Loss" dataDxfId="12"/>
-    <tableColumn id="7" xr3:uid="{6A4DE3F1-C938-44DE-99B9-0B1E0FA24873}" name="Epoch" dataDxfId="11"/>
+    <tableColumn id="1" xr3:uid="{6DA5A62F-F191-4700-A4DA-1ECCC0798408}" name="Dataset Name" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{6229C568-365F-4FB5-B5A5-14F4C8640478}" name="Accuracy" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{75BF09EF-9AEE-4394-90C3-0A038B9B0213}" name="Precision" dataDxfId="13"/>
+    <tableColumn id="4" xr3:uid="{4B15F953-1DB4-400F-816B-C322B01A4C96}" name="Recall" dataDxfId="12"/>
+    <tableColumn id="5" xr3:uid="{F8BED74C-48BE-4570-B328-816EDC50C33B}" name="F1" dataDxfId="11"/>
+    <tableColumn id="6" xr3:uid="{09327258-5F58-4797-9AC7-3B966B9FB96D}" name="Loss" dataDxfId="10"/>
+    <tableColumn id="7" xr3:uid="{6A4DE3F1-C938-44DE-99B9-0B1E0FA24873}" name="Epoch" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{C5F7CB90-1779-45BE-B45B-8B2C1DA5ED85}" name="Table7" displayName="Table7" ref="J3:P5" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{C5F7CB90-1779-45BE-B45B-8B2C1DA5ED85}" name="Table7" displayName="Table7" ref="J3:P5" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
   <autoFilter ref="J3:P5" xr:uid="{C5F7CB90-1779-45BE-B45B-8B2C1DA5ED85}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{3CC08680-A79C-4D27-BE3D-6AE070823B8C}" name="Model" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{3C682DE3-7736-4A52-B9FC-C672D5C975DF}" name="Accuracy" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{A74316B3-E6F0-4C17-9EED-3CB3BE551060}" name="Precision" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{4C15B6E3-3786-4187-9279-E2B32A9494B0}" name="Recall" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{75FC2AAE-9384-49C8-B4E7-3A4E7C604883}" name="F1" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{E499D22F-E3E7-4635-A303-F22CDB256B1A}" name="Loss" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{130339A0-B416-400E-814E-9CB19808E804}" name="Epoch" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{3CC08680-A79C-4D27-BE3D-6AE070823B8C}" name="Model" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{3C682DE3-7736-4A52-B9FC-C672D5C975DF}" name="Accuracy" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{A74316B3-E6F0-4C17-9EED-3CB3BE551060}" name="Precision" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{4C15B6E3-3786-4187-9279-E2B32A9494B0}" name="Recall" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{75FC2AAE-9384-49C8-B4E7-3A4E7C604883}" name="F1" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{E499D22F-E3E7-4635-A303-F22CDB256B1A}" name="Loss" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{130339A0-B416-400E-814E-9CB19808E804}" name="Epoch" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1135,30 +1144,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{106E9688-4ED0-4B67-B55A-23F33FEBEBE2}">
   <dimension ref="B2:P28"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="3"/>
-    <col min="2" max="2" width="28.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.28515625" style="3" customWidth="1"/>
-    <col min="4" max="4" width="10.5703125" style="3" customWidth="1"/>
-    <col min="5" max="9" width="9.140625" style="3"/>
-    <col min="10" max="10" width="10.5703125" style="3" customWidth="1"/>
+    <col min="1" max="1" width="9.1640625" style="3"/>
+    <col min="2" max="2" width="28.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.33203125" style="3" customWidth="1"/>
+    <col min="4" max="4" width="10.5" style="3" customWidth="1"/>
+    <col min="5" max="9" width="9.1640625" style="3"/>
+    <col min="10" max="10" width="24.83203125" style="3" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11" style="3" customWidth="1"/>
-    <col min="12" max="12" width="10.85546875" style="3" customWidth="1"/>
-    <col min="13" max="15" width="10.5703125" style="3" customWidth="1"/>
-    <col min="16" max="16384" width="9.140625" style="3"/>
+    <col min="12" max="12" width="10.83203125" style="3" customWidth="1"/>
+    <col min="13" max="15" width="10.5" style="3" customWidth="1"/>
+    <col min="16" max="16384" width="9.1640625" style="3"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B2" s="2" t="s">
+    <row r="2" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="B2" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="2"/>
-      <c r="J2" s="4" t="s">
+      <c r="C2" s="7"/>
+      <c r="J2" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
@@ -1202,7 +1211,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B4" s="3" t="s">
         <v>2</v>
       </c>
@@ -1246,26 +1255,26 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B5" s="5" t="s">
+    <row r="5" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="B5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="4">
         <v>0.94199999999999995</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="4">
         <v>0.91009287368524705</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="4">
         <v>0.92115560716326905</v>
       </c>
-      <c r="F5" s="5">
+      <c r="F5" s="4">
         <v>0.91533564022587399</v>
       </c>
-      <c r="G5" s="5">
+      <c r="G5" s="4">
         <v>0.191635861992836</v>
       </c>
-      <c r="H5" s="5">
+      <c r="H5" s="4">
         <v>3</v>
       </c>
       <c r="J5" s="3" t="s">
@@ -1290,53 +1299,53 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B6" s="5" t="s">
+    <row r="6" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="B6" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="5">
+      <c r="C6" s="4">
         <v>0.94199999999999995</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="4">
         <v>0.91009287368524705</v>
       </c>
-      <c r="E6" s="5">
+      <c r="E6" s="4">
         <v>0.92115560716326905</v>
       </c>
-      <c r="F6" s="5">
+      <c r="F6" s="4">
         <v>0.91533564022587399</v>
       </c>
-      <c r="G6" s="5">
+      <c r="G6" s="4">
         <v>0.191635861992836</v>
       </c>
-      <c r="H6" s="5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B7" s="5" t="s">
+      <c r="H6" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="B7" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="4">
         <v>0.94199999999999995</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="4">
         <v>0.91009287368524705</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="4">
         <v>0.92115560716326905</v>
       </c>
-      <c r="F7" s="5">
+      <c r="F7" s="4">
         <v>0.91533564022587399</v>
       </c>
-      <c r="G7" s="5">
+      <c r="G7" s="4">
         <v>0.191635861992836</v>
       </c>
-      <c r="H7" s="5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="H7" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B8" s="3" t="s">
         <v>16</v>
       </c>
@@ -1359,59 +1368,59 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B9" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="7">
+      <c r="C9" s="6">
         <v>0.9355</v>
       </c>
-      <c r="D9" s="7">
+      <c r="D9" s="6">
         <v>0.90203298486156802</v>
       </c>
-      <c r="E9" s="7">
+      <c r="E9" s="6">
         <v>0.90715039969428501</v>
       </c>
-      <c r="F9" s="7">
+      <c r="F9" s="6">
         <v>0.90403925299948695</v>
       </c>
-      <c r="G9" s="7">
+      <c r="G9" s="6">
         <v>0.47319608926772999</v>
       </c>
       <c r="H9" s="3">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B10" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C10" s="7">
+      <c r="C10" s="6">
         <v>0.94799999999999995</v>
       </c>
-      <c r="D10" s="7">
+      <c r="D10" s="6">
         <v>0.94802861178020803</v>
       </c>
-      <c r="E10" s="7">
+      <c r="E10" s="6">
         <v>0.94798241355127499</v>
       </c>
-      <c r="F10" s="7">
+      <c r="F10" s="6">
         <v>0.94790593102700604</v>
       </c>
-      <c r="G10" s="7">
+      <c r="G10" s="6">
         <v>0.37256675958633401</v>
       </c>
       <c r="H10" s="3">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="J11" s="4" t="s">
+    <row r="11" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="J11" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="K11" s="4"/>
-    </row>
-    <row r="12" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="K11" s="2"/>
+    </row>
+    <row r="12" spans="2:16" x14ac:dyDescent="0.2">
       <c r="J12" s="3" t="s">
         <v>1</v>
       </c>
@@ -1434,7 +1443,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:16" x14ac:dyDescent="0.2">
       <c r="J13" s="3" t="s">
         <v>2</v>
       </c>
@@ -1457,76 +1466,79 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="J14" s="5" t="s">
+    <row r="14" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="J14" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="K14" s="6">
+      <c r="K14" s="5">
         <v>0.93700000000000006</v>
       </c>
-      <c r="L14" s="6">
+      <c r="L14" s="5">
         <v>0.92557082683330705</v>
       </c>
-      <c r="M14" s="6">
+      <c r="M14" s="5">
         <v>0.90349649643238195</v>
       </c>
-      <c r="N14" s="6">
+      <c r="N14" s="5">
         <v>0.91098762484752904</v>
       </c>
-      <c r="O14" s="6">
+      <c r="O14" s="5">
         <v>0.17923152446746801</v>
       </c>
-      <c r="P14" s="5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="15" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="J15" s="5" t="s">
+      <c r="P14" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="J15" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K15" s="6">
+      <c r="K15" s="5">
         <v>0.93700000000000006</v>
       </c>
-      <c r="L15" s="6">
+      <c r="L15" s="5">
         <v>0.92557082683330705</v>
       </c>
-      <c r="M15" s="6">
+      <c r="M15" s="5">
         <v>0.90349649643238195</v>
       </c>
-      <c r="N15" s="6">
+      <c r="N15" s="5">
         <v>0.91098762484752904</v>
       </c>
-      <c r="O15" s="6">
+      <c r="O15" s="5">
         <v>0.17923152446746801</v>
       </c>
-      <c r="P15" s="5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="16" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="J16" s="5" t="s">
+      <c r="P15" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="J16" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="K16" s="6">
+      <c r="K16" s="5">
         <v>0.93700000000000006</v>
       </c>
-      <c r="L16" s="6">
+      <c r="L16" s="5">
         <v>0.92557082683330705</v>
       </c>
-      <c r="M16" s="6">
+      <c r="M16" s="5">
         <v>0.90349649643238195</v>
       </c>
-      <c r="N16" s="6">
+      <c r="N16" s="5">
         <v>0.91098762484752904</v>
       </c>
-      <c r="O16" s="6">
+      <c r="O16" s="5">
         <v>0.17923152446746801</v>
       </c>
-      <c r="P16" s="5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="P16" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="H17" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="J17" s="3" t="s">
         <v>16</v>
       </c>
@@ -1549,13 +1561,50 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B20" s="4" t="s">
+    <row r="18" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="H18" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="J18" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="P18" s="3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="H19" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J19" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="K19" s="3">
+        <v>0.95750000000000002</v>
+      </c>
+      <c r="L19" s="3">
+        <v>0.95820000000000005</v>
+      </c>
+      <c r="M19" s="3">
+        <v>0.95740000000000003</v>
+      </c>
+      <c r="N19" s="3">
+        <v>0.95730000000000004</v>
+      </c>
+      <c r="O19" s="3">
+        <v>0.25230000000000002</v>
+      </c>
+      <c r="P19" s="3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="B20" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="4"/>
-    </row>
-    <row r="21" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="C20" s="2"/>
+    </row>
+    <row r="21" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B21" s="3" t="s">
         <v>1</v>
       </c>
@@ -1578,7 +1627,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="22" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B22" s="3" t="s">
         <v>2</v>
       </c>
@@ -1601,76 +1650,76 @@
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B23" s="5" t="s">
+    <row r="23" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="B23" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C23" s="6">
+      <c r="C23" s="5">
         <v>0.94299999999999995</v>
       </c>
-      <c r="D23" s="6">
+      <c r="D23" s="5">
         <v>0.917014698774683</v>
       </c>
-      <c r="E23" s="6">
+      <c r="E23" s="5">
         <v>0.91827723390579796</v>
       </c>
-      <c r="F23" s="6">
+      <c r="F23" s="5">
         <v>0.917529975022639</v>
       </c>
-      <c r="G23" s="6">
+      <c r="G23" s="5">
         <v>0.18735474348068201</v>
       </c>
-      <c r="H23" s="5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="24" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B24" s="5" t="s">
+      <c r="H23" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="B24" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C24" s="6">
+      <c r="C24" s="5">
         <v>0.94299999999999995</v>
       </c>
-      <c r="D24" s="6">
+      <c r="D24" s="5">
         <v>0.917014698774683</v>
       </c>
-      <c r="E24" s="6">
+      <c r="E24" s="5">
         <v>0.91827723390579796</v>
       </c>
-      <c r="F24" s="6">
+      <c r="F24" s="5">
         <v>0.917529975022639</v>
       </c>
-      <c r="G24" s="6">
+      <c r="G24" s="5">
         <v>0.18735474348068201</v>
       </c>
-      <c r="H24" s="5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="25" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B25" s="5" t="s">
+      <c r="H24" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="B25" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C25" s="6">
+      <c r="C25" s="5">
         <v>0.94299999999999995</v>
       </c>
-      <c r="D25" s="6">
+      <c r="D25" s="5">
         <v>0.917014698774683</v>
       </c>
-      <c r="E25" s="6">
+      <c r="E25" s="5">
         <v>0.91827723390579796</v>
       </c>
-      <c r="F25" s="6">
+      <c r="F25" s="5">
         <v>0.917529975022639</v>
       </c>
-      <c r="G25" s="6">
+      <c r="G25" s="5">
         <v>0.18735474348068201</v>
       </c>
-      <c r="H25" s="5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="26" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="H25" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B26" s="3" t="s">
         <v>16</v>
       </c>
@@ -1693,7 +1742,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B27" s="3" t="s">
         <v>18</v>
       </c>
@@ -1716,7 +1765,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="28" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B28" s="3" t="s">
         <v>2</v>
       </c>

</xml_diff>